<commit_message>
Add categorization columns and fix missing actual outputs for last 3 test cases
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +115,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,15 +462,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="49.95" customHeight="1"/>
   <cols>
     <col width="10.88671875" customWidth="1" min="1" max="1"/>
     <col width="22.109375" customWidth="1" min="3" max="3"/>
     <col width="25.33203125" customWidth="1" min="4" max="4"/>
     <col width="22.5546875" customWidth="1" min="5" max="5"/>
-    <col width="14.33203125" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
     <col width="12.33203125" customWidth="1" min="9" max="10"/>
   </cols>
   <sheetData>
@@ -502,6 +505,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Singlish input types covered</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Evidence or rationale for the input type covered</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="79.95" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -534,6 +547,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as wune, mokada inserted</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="79.95" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -566,6 +589,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as hondatama, eya inserted; Rationale: Consecutive English words such as "oyage ammata kohomada"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="79.95" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -588,10 +621,24 @@
           <t>ඒක බලාපු උඩ කියාපන්.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as uda, kiyapan inserted; Rationale: Consecutive English words such as "eka balapu uda"</t>
         </is>
       </c>
     </row>
@@ -626,6 +673,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as karapan, wahama inserted; Rationale: Consecutive English words such as "wahama mama kiwwa"; Rationale: Contains time format; Rationale: Includes words such as api</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="79.95" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -658,6 +715,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as !, ?; Rationale: Single words such as bohoma, machan inserted; Rationale: Consecutive English words such as "bohoma kala nathara"; Rationale: Includes slang such as machan</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="79.95" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -690,6 +757,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as !; Rationale: Single words such as Oyata, subhapathum inserted; Rationale: Consecutive English words such as "Subha dawasak wewa"</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="79.95" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -722,6 +799,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as katha, poddak inserted; Rationale: Consecutive English words such as "mama api gena"; Rationale: Includes slang such as thiyanawa; Rationale: Contains time format; Rationale: Includes words such as api</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="79.95" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -754,6 +841,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as enna, gate inserted; Rationale: Consecutive English words such as "mama enna kalin"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="49.95" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -786,6 +883,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as dannne, nehe inserted; Rationale: Consecutive English words such as "mama dannne nehe"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="49.95" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -818,6 +925,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as gena, nehe inserted; Rationale: Consecutive English words such as "mama e gena"; Rationale: Includes slang such as machan; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="49.95" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -850,6 +967,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as katha, manda inserted; Rationale: Consecutive English words such as "manda manda katha"; Rationale: Includes words such as api</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="49.95" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -882,6 +1009,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as poddak, Poddak inserted; Rationale: Consecutive English words such as "Poddak poddak kiyapan"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="49.95" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -914,6 +1051,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as !, ?; Rationale: Single words such as me, ado inserted; Rationale: Consecutive English words such as "oya me kiwweda"; Rationale: Includes slang such as ado</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="49.95" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -946,6 +1093,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as hm, mata inserted; Rationale: Consecutive English words such as "mata therenne nehe"</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="49.95" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -978,6 +1135,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as enna, nathnam inserted; Rationale: Consecutive English words such as "man heta enna"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="49.95" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1000,10 +1167,24 @@
           <t>මොකක්ද අපි කරන්නේ? මගේ හදාපු plan එක වැරදි වේලා.</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as hdapu, karanne inserted; Rationale: Consecutive English words such as "mokakd api karanne"; Rationale: Includes words such as api</t>
         </is>
       </c>
     </row>
@@ -1028,10 +1209,24 @@
           <t>මම අද school එකේ project එක finish කරලා ගියා.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as school, eke inserted; Rationale: Consecutive English words such as "mama ada school"; Rationale: Contains time format</t>
         </is>
       </c>
     </row>
@@ -1056,10 +1251,24 @@
           <t>ඔය අද free ද? අපි lunch ගන්න යනවද?</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as free, ganna inserted; Rationale: Consecutive English words such as "oya ada free"; Rationale: Includes words such as api</t>
         </is>
       </c>
     </row>
@@ -1084,10 +1293,24 @@
           <t>මම හෙට out of office, so call me only if urgent.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as out, so inserted; Rationale: Consecutive English words such as "mama heta out"; Rationale: Contains time format</t>
         </is>
       </c>
     </row>
@@ -1112,10 +1335,24 @@
           <t>meeting එක cancel වේලා, so we need to reschedule ASAP.</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as ASAP, so inserted; Rationale: Consecutive English words such as "meeting eka cancel"</t>
         </is>
       </c>
     </row>
@@ -1140,10 +1377,24 @@
           <t>ඔය screenshot එක ගත්තද? මට send කරන්න.</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as gathada, karanna inserted; Rationale: Consecutive English words such as "oya screenshot eka"</t>
         </is>
       </c>
     </row>
@@ -1178,6 +1429,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, Platform/App names in Singlish</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as karala, karannm inserted; Rationale: Consecutive English words such as "mama eka Google"; Rationale: Contains time format; Rationale: Includes google</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="49.95" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1210,6 +1471,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as awe, Netflix inserted; Rationale: Consecutive English words such as "Netflix eke new"</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="49.95" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1242,6 +1513,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, Platform/App names in Singlish</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as post, karanda inserted; Rationale: Consecutive English words such as "Instagram story eka"; Rationale: Contains time format; Rationale: Includes instagram</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="49.95" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -1274,6 +1555,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as kiyanne, submit inserted; Rationale: Consecutive English words such as "HR kiyanne oya"</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="49.95" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1306,6 +1597,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as eke, api inserted; Rationale: Consecutive English words such as "api GPS eke"; Rationale: Includes words such as api</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="49.95" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -1328,10 +1629,24 @@
           <t>මම හෙට uni එකේ presentation එකක් තියනවා, nervous wage.</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as eke, uni inserted; Rationale: Consecutive English words such as "mama heta uni"; Rationale: Includes slang such as thiyanawa; Rationale: Contains time format</t>
         </is>
       </c>
     </row>
@@ -1356,10 +1671,24 @@
           <t>doc කියන්නේ op කාලා පසේ rest ගන්න කියලා.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as rest, kiyanne inserted; Rationale: Consecutive English words such as "doc kiyanne op"</t>
         </is>
       </c>
     </row>
@@ -1394,6 +1723,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as walata, api inserted; Rationale: Consecutive English words such as "api Kandy walata"; Rationale: Includes words such as api</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="49.95" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -1426,6 +1765,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as Arcade, gihilla inserted; Rationale: Consecutive English words such as "walata gihilla Arcade"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="49.95" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -1458,6 +1807,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as match, eke inserted; Rationale: Consecutive English words such as "Chamari aiye match"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="49.95" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -1490,6 +1849,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as saha, interview inserted; Rationale: Consecutive English words such as "Nuwan saha Kasun"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="49.95" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -1522,6 +1891,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as hadagaththa, giyama inserted; Rationale: Consecutive English words such as "dawase giyama eka"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="49.95" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -1544,10 +1923,24 @@
           <t>අපි 3rd floor එකේ කාමර 5ක් දේකා ගියා.</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as kamara, eke inserted; Rationale: Consecutive English words such as "floor eke kamara"; Rationale: Contains time format; Rationale: Includes words such as api</t>
         </is>
       </c>
     </row>
@@ -1572,10 +1965,24 @@
           <t>ඒ jacket එක LKR 4500 ලා ගෙදා, worthd?</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ?; Rationale: Single words such as worthda, gedda inserted; Rationale: Consecutive English words such as "e jacket eka"</t>
         </is>
       </c>
     </row>
@@ -1600,10 +2007,24 @@
           <t>USD 50 කියන්නේ රුපියල් වලින් කොච්චරද අද?</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as kiyanne, walin inserted; Rationale: Consecutive English words such as "kiyanne rupiyel walin"</t>
         </is>
       </c>
     </row>
@@ -1628,10 +2049,24 @@
           <t>අපි හෙට 8:00AM ට ගෑත්වේනා ඒක හොඳයි.</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ., :; Rationale: Single words such as hondai, api inserted; Rationale: Consecutive English words such as "ta gathwena eka"; Rationale: Contains time format; Rationale: Includes words such as api</t>
         </is>
       </c>
     </row>
@@ -1666,6 +2101,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as late, start inserted; Rationale: Consecutive English words such as "walata start wenawa"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="49.95" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -1698,6 +2143,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as March, kiyala inserted; Rationale: Consecutive English words such as "submission deadline eka"</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="49.95" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -1730,6 +2185,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as thiyenawa, eka inserted; Rationale: Consecutive English words such as "ta schedule karala"; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="49.95" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -1762,6 +2227,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., ?; Rationale: Single words such as thiyenawa, e inserted; Rationale: Consecutive English words such as "e fabric eka"</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="49.95" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -1794,6 +2269,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as temperature, newath inserted; Rationale: Consecutive English words such as "dengue newath penne"; Rationale: Includes slang such as thiyanawa</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="49.95" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -1826,6 +2311,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as puka, kiyala inserted; Rationale: Consecutive English words such as "uba puka hedda"; Rationale: Includes slang such as bro</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="49.95" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -1858,6 +2353,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as sira, ekka inserted; Rationale: Consecutive English words such as "ada sira dawasak"</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="49.95" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -1890,6 +2395,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, Platform/App names in Singlish</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., :, ?; Rationale: Single words such as post, eke inserted; Rationale: Consecutive English words such as "mama comment dammada"; Rationale: Contains time format; Rationale: Includes facebook</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="49.95" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -1922,6 +2437,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., :, ?; Rationale: Single words such as me, eke inserted; Rationale: Consecutive English words such as "oya me group"; Rationale: Includes slang such as bro; Rationale: Contains time format</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="49.95" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -1954,6 +2479,16 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as dannawada, skip inserted; Rationale: Consecutive English words such as "ada class skip"</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="49.95" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -1976,10 +2511,24 @@
           <t>finally results ආවේ 🎉 මම pass වේලා 😭 ගොඩක් happy.</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr"/>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as awe, results inserted; Rationale: Consecutive English words such as "finally results awe"; Rationale: Contains time format; Rationale: Includes words such as app</t>
         </is>
       </c>
     </row>
@@ -2004,10 +2553,24 @@
           <t>මචං, ඔය දන්නවාද API එක test කරන්න best tool එකක්? මම Postman use කරලා තියෙනවා, bat proper automation එකක් හදන්න ඕනේ. ඔයාට කිසි idea එකක් තියෙනවාද? මම හෙට meeting එකට late වෙනවා නිසා අද එවන්න බෑ.</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats, English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., ?; Rationale: Single words such as Postman, proper inserted; Rationale: Consecutive English words such as "oya dannawada API"; Rationale: Includes slang such as machan, thiyanawa; Rationale: Contains time format; Rationale: Includes words such as api</t>
         </is>
       </c>
     </row>
@@ -2032,10 +2595,24 @@
           <t>අඩෝ නං, මම අද 9:00AM ට office ගියා. HR කිව්වා IT team එකට new laptop 2 දාපු කියලා. Budget එක LKR 150,000 කියලා කිව්වා. මම හෙට බලාගන්නා ඕනේ කොච්චරට order කරන්නා ඕනේ කියලා. ඔය help කරන්ද පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr"/>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>No conversion output</t>
+        </is>
+      </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
           <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., :, ?; Rationale: Single words such as Mama, dapu inserted; Rationale: Consecutive English words such as "ta office giya"; Rationale: Includes slang such as ado, puluwanda; Rationale: Contains time format</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add detailed evidence and rationale for all 50 test case categorizations
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -469,8 +469,8 @@
     <col width="22.109375" customWidth="1" min="3" max="3"/>
     <col width="25.33203125" customWidth="1" min="4" max="4"/>
     <col width="22.5546875" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
     <col width="12.33203125" customWidth="1" min="9" max="10"/>
   </cols>
   <sheetData>
@@ -549,12 +549,14 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as wune, mokada inserted</t>
+          <t>Evidence: "mokada wune?"
+Rationale: It uses punctuation such as ?
+Rationale: Single words such as 'mokada, wune' are inserted in between Singlish text</t>
         </is>
       </c>
     </row>
@@ -591,12 +593,16 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as hondatama, eya inserted; Rationale: Consecutive English words such as "oyage ammata kohomada"; Rationale: Contains time format</t>
+          <t>Evidence: "oyage ammata kohomada?"
+Rationale: It uses punctuation such as ?
+Rationale: Single words such as 'oyage, ammata, kohomada, eya' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "oyage ammata kohomada" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -633,12 +639,14 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as uda, kiyapan inserted; Rationale: Consecutive English words such as "eka balapu uda"</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'eka, balapu, uda, kiyapan' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "eka balapu uda" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -675,12 +683,17 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as karapan, wahama inserted; Rationale: Consecutive English words such as "wahama mama kiwwa"; Rationale: Contains time format; Rationale: Includes words such as api</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'wahama, mama, kiwwa, deyak' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "wahama mama kiwwa" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'
+Rationale: Input includes 'am'
+Rationale: Input includes 'nehe'</t>
         </is>
       </c>
     </row>
@@ -717,12 +730,16 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as !, ?; Rationale: Single words such as bohoma, machan inserted; Rationale: Consecutive English words such as "bohoma kala nathara"; Rationale: Includes slang such as machan</t>
+          <t>Evidence: "kohomada machan?"
+Rationale: It uses punctuation such as !, ?
+Rationale: Single words such as 'kohomada, machan, bohoma, kala' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "bohoma kala nathara" is inserted inside the Singlish input
+Rationale: Input includes 'machan'</t>
         </is>
       </c>
     </row>
@@ -759,12 +776,14 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as !; Rationale: Single words such as Oyata, subhapathum inserted; Rationale: Consecutive English words such as "Subha dawasak wewa"</t>
+          <t>Rationale: It uses punctuation such as !
+Rationale: Single words such as 'Subha, dawasak, wewa, Oyata' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "Subha dawasak wewa" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -801,12 +820,17 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as katha, poddak inserted; Rationale: Consecutive English words such as "mama api gena"; Rationale: Includes slang such as thiyanawa; Rationale: Contains time format; Rationale: Includes words such as api</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'poddak, inna, mama, api' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama api gena" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'
+Rationale: Input includes 'am'
+Rationale: Input includes 'thiyanawa'</t>
         </is>
       </c>
     </row>
@@ -843,12 +867,15 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as enna, gate inserted; Rationale: Consecutive English words such as "mama enna kalin"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'mama, enna, kalin, gate' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama enna kalin" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -885,12 +912,16 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as dannne, nehe inserted; Rationale: Consecutive English words such as "mama dannne nehe"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'nehe, mama, dannne' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama dannne nehe" is inserted inside the Singlish input
+Rationale: Input includes 'am'
+Rationale: Input includes 'nehe'</t>
         </is>
       </c>
     </row>
@@ -927,12 +958,17 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+          <t>Requests, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as gena, nehe inserted; Rationale: Consecutive English words such as "mama e gena"; Rationale: Includes slang such as machan; Rationale: Contains time format</t>
+          <t>Evidence: "we nehe. Godak thanks machan."
+Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'Aiyo, mama, gena, hithuwe' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama e gena" is inserted inside the Singlish input
+Rationale: Input includes 'am'
+Rationale: Input includes 'machan, nehe'</t>
         </is>
       </c>
     </row>
@@ -969,12 +1005,15 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as katha, manda inserted; Rationale: Consecutive English words such as "manda manda katha"; Rationale: Includes words such as api</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'manda, katha, karanna, epa' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "manda manda katha" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1050,15 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as poddak, Poddak inserted; Rationale: Consecutive English words such as "Poddak poddak kiyapan"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'Poddak, poddak, kiyapan, mama' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "Poddak poddak kiyapan" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1053,12 +1095,16 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as !, ?; Rationale: Single words such as me, ado inserted; Rationale: Consecutive English words such as "oya me kiwweda"; Rationale: Includes slang such as ado</t>
+          <t>Evidence: "ado!! oya me kiwweda?"
+Rationale: It uses punctuation such as !, ?
+Rationale: Single words such as 'ado, oya, me, kiwweda' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "oya me kiwweda" is inserted inside the Singlish input
+Rationale: Input includes 'ado'</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1141,15 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as hm, mata inserted; Rationale: Consecutive English words such as "mata therenne nehe"</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'hm, mata, therenne, nehe' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mata therenne nehe" is inserted inside the Singlish input
+Rationale: Input includes 'nehe'</t>
         </is>
       </c>
     </row>
@@ -1137,12 +1186,15 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as enna, nathnam inserted; Rationale: Consecutive English words such as "man heta enna"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'man, heta, enna, hithn' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "man heta enna" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1179,12 +1231,16 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as hdapu, karanne inserted; Rationale: Consecutive English words such as "mokakd api karanne"; Rationale: Includes words such as api</t>
+          <t>Evidence: "mokakd api karanne?"
+Rationale: It uses punctuation such as ., ?
+Rationale: Single words such as 'mokakd, api, karanne, mage' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mokakd api karanne" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'</t>
         </is>
       </c>
     </row>
@@ -1221,12 +1277,15 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as school, eke inserted; Rationale: Consecutive English words such as "mama ada school"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'mama, ada, school, eke' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama ada school" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1263,12 +1322,16 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as free, ganna inserted; Rationale: Consecutive English words such as "oya ada free"; Rationale: Includes words such as api</t>
+          <t>Evidence: "oya ada free da?"
+Rationale: It uses punctuation such as ?
+Rationale: Single words such as 'oya, ada, free, da' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "oya ada free" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'</t>
         </is>
       </c>
     </row>
@@ -1305,12 +1368,15 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as out, so inserted; Rationale: Consecutive English words such as "mama heta out"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'mama, heta, out, of' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama heta out" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1413,14 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as ASAP, so inserted; Rationale: Consecutive English words such as "meeting eka cancel"</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'meeting, eka, cancel, wela' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "meeting eka cancel" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -1389,12 +1457,15 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as gathada, karanna inserted; Rationale: Consecutive English words such as "oya screenshot eka"</t>
+          <t>Evidence: "oya screenshot eka gathada?"
+Rationale: It uses punctuation such as ., ?
+Rationale: Single words such as 'oya, screenshot, eka, gathada' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "oya screenshot eka" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -1431,12 +1502,17 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, Platform/App names in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Platform/App Names in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as karala, karannm inserted; Rationale: Consecutive English words such as "mama eka Google"; Rationale: Contains time format; Rationale: Includes google</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'mama, eka, Google, Drive' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama eka Google" is inserted inside the Singlish input
+Rationale: Input includes words such as 'link'
+Rationale: Input includes words such as 'google'
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1473,12 +1549,15 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Platform/App Names in Singlish</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as awe, Netflix inserted; Rationale: Consecutive English words such as "Netflix eke new"</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'Netflix, eke, new, season' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "Netflix eke new" is inserted inside the Singlish input
+Rationale: Input includes words such as 'netflix'</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1594,17 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, Platform/App names in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Platform/App Names in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as post, karanda inserted; Rationale: Consecutive English words such as "Instagram story eka"; Rationale: Contains time format; Rationale: Includes instagram</t>
+          <t>Evidence: "Instagram story eka post karanda?"
+Rationale: It uses punctuation such as ., ?
+Rationale: Single words such as 'Instagram, story, eka, post' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "Instagram story eka" is inserted inside the Singlish input
+Rationale: Input includes words such as 'instagram'
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1557,12 +1641,14 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as kiyanne, submit inserted; Rationale: Consecutive English words such as "HR kiyanne oya"</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'HR, kiyanne, oya, CV' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "HR kiyanne oya" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1685,16 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., ?; Rationale: Single words such as eke, api inserted; Rationale: Consecutive English words such as "api GPS eke"; Rationale: Includes words such as api</t>
+          <t>Evidence: "ETA kohomada?"
+Rationale: It uses punctuation such as ., ?
+Rationale: Single words such as 'ETA, kohomada, api, GPS' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "api GPS eke" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1731,16 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as eke, uni inserted; Rationale: Consecutive English words such as "mama heta uni"; Rationale: Includes slang such as thiyanawa; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'mama, heta, uni, eke' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama heta uni" is inserted inside the Singlish input
+Rationale: Input includes 'am'
+Rationale: Input includes 'thiyanawa'</t>
         </is>
       </c>
     </row>
@@ -1683,12 +1777,14 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as rest, kiyanne inserted; Rationale: Consecutive English words such as "doc kiyanne op"</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'doc, kiyanne, op, kala' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "doc kiyanne op" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -1725,12 +1821,15 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as walata, api inserted; Rationale: Consecutive English words such as "api Kandy walata"; Rationale: Includes words such as api</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'api, Kandy, walata, giya' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "api Kandy walata" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'</t>
         </is>
       </c>
     </row>
@@ -1767,12 +1866,15 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as Arcade, gihilla inserted; Rationale: Consecutive English words such as "walata gihilla Arcade"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'heta, Colombo, walata, gihilla' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "walata gihilla Arcade" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1809,12 +1911,15 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as match, eke inserted; Rationale: Consecutive English words such as "Chamari aiye match"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'Chamari, aiye, match, eke' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "Chamari aiye match" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1851,12 +1956,15 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as saha, interview inserted; Rationale: Consecutive English words such as "Nuwan saha Kasun"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'Nuwan, saha, Kasun, dennama' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "Nuwan saha Kasun" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1893,12 +2001,15 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as hadagaththa, giyama inserted; Rationale: Consecutive English words such as "dawase giyama eka"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'mama, dawase, giyama, eka' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "dawase giyama eka" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1935,12 +2046,16 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as kamara, eke inserted; Rationale: Consecutive English words such as "floor eke kamara"; Rationale: Contains time format; Rationale: Includes words such as api</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'api, floor, eke, kamara' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "floor eke kamara" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -1977,12 +2092,16 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ?; Rationale: Single words such as worthda, gedda inserted; Rationale: Consecutive English words such as "e jacket eka"</t>
+          <t>Evidence: "e jacket eka LKR 4500 la gedda, worthda?"
+Rationale: It uses punctuation such as ,, ?
+Rationale: Single words such as 'jacket, eka, LKR, la' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "e jacket eka" is inserted inside the Singlish input
+Rationale: Input includes 'gedda'</t>
         </is>
       </c>
     </row>
@@ -2019,12 +2138,15 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ?; Rationale: Single words such as kiyanne, walin inserted; Rationale: Consecutive English words such as "kiyanne rupiyel walin"</t>
+          <t>Evidence: "USD 50 kiyanne rupiyel walin kochcharada ada?"
+Rationale: It uses punctuation such as ?
+Rationale: Single words such as 'USD, kiyanne, rupiyel, walin' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "kiyanne rupiyel walin" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -2061,12 +2183,16 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ., :; Rationale: Single words such as hondai, api inserted; Rationale: Consecutive English words such as "ta gathwena eka"; Rationale: Contains time format; Rationale: Includes words such as api</t>
+          <t>Rationale: It uses punctuation such as ., :
+Rationale: Single words such as 'api, heta, ta, gathwena' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "ta gathwena eka" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'
+Rationale: Input includes '8:00'</t>
         </is>
       </c>
     </row>
@@ -2103,12 +2229,15 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as late, start inserted; Rationale: Consecutive English words such as "walata start wenawa"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'class, eka, walata, start' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "walata start wenawa" is inserted inside the Singlish input
+Rationale: Input includes '30pm'</t>
         </is>
       </c>
     </row>
@@ -2145,12 +2274,14 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as March, kiyala inserted; Rationale: Consecutive English words such as "submission deadline eka"</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'submission, deadline, eka, March' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "submission deadline eka" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -2187,12 +2318,15 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as thiyenawa, eka inserted; Rationale: Consecutive English words such as "ta schedule karala"; Rationale: Contains time format</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'exam, eka, ta, schedule' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "ta schedule karala" is inserted inside the Singlish input
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -2229,12 +2363,15 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., ?; Rationale: Single words such as thiyenawa, e inserted; Rationale: Consecutive English words such as "e fabric eka"</t>
+          <t>Evidence: "e fabric eka meter 2.5k thiyenawa, poruwa?"
+Rationale: It uses punctuation such as ,, ., ?
+Rationale: Single words such as 'fabric, eka, meter, thiyenawa' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "e fabric eka" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -2271,12 +2408,15 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as temperature, newath inserted; Rationale: Consecutive English words such as "dengue newath penne"; Rationale: Includes slang such as thiyanawa</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'dengue, newath, penne, temperature' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "dengue newath penne" is inserted inside the Singlish input
+Rationale: Input includes 'thiyanawa'</t>
         </is>
       </c>
     </row>
@@ -2313,12 +2453,15 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as puka, kiyala inserted; Rationale: Consecutive English words such as "uba puka hedda"; Rationale: Includes slang such as bro</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'bro, uba, puka, hedda' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "uba puka hedda" is inserted inside the Singlish input
+Rationale: Input includes 'bro'</t>
         </is>
       </c>
     </row>
@@ -2355,12 +2498,14 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as ,, .; Rationale: Single words such as sira, ekka inserted; Rationale: Consecutive English words such as "ada sira dawasak"</t>
+          <t>Rationale: It uses punctuation such as ,, .
+Rationale: Single words such as 'ada, sira, dawasak, ekka' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "ada sira dawasak" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -2397,12 +2542,17 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, Platform/App names in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Platform/App Names in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ., :, ?; Rationale: Single words such as post, eke inserted; Rationale: Consecutive English words such as "mama comment dammada"; Rationale: Contains time format; Rationale: Includes facebook</t>
+          <t>Evidence: "mama comment dammada oya Facebook post eke?"
+Rationale: It uses punctuation such as ., :, ?
+Rationale: Single words such as 'mama, comment, dammada, oya' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "mama comment dammada" is inserted inside the Singlish input
+Rationale: Input includes words such as 'facebook'
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -2439,12 +2589,17 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., :, ?; Rationale: Single words such as me, eke inserted; Rationale: Consecutive English words such as "oya me group"; Rationale: Includes slang such as bro; Rationale: Contains time format</t>
+          <t>Evidence: "@Malith bro, oya me group eke admin da?"
+Rationale: It uses punctuation such as ,, ., :, ?
+Rationale: Single words such as 'Malith, bro, oya, me' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "oya me group" is inserted inside the Singlish input
+Rationale: Input includes 'am'
+Rationale: Input includes 'bro'</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2636,14 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as dannawada, skip inserted; Rationale: Consecutive English words such as "ada class skip"</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'ada, class, skip, karala' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "ada class skip" is inserted inside the Singlish input</t>
         </is>
       </c>
     </row>
@@ -2523,12 +2680,16 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with time formats, English digital terms in Singlish</t>
+          <t>Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>Rationale: Uses punctuation such as .; Rationale: Single words such as awe, results inserted; Rationale: Consecutive English words such as "finally results awe"; Rationale: Contains time format; Rationale: Includes words such as app</t>
+          <t>Rationale: It uses punctuation such as .
+Rationale: Single words such as 'finally, results, awe, mama' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "finally results awe" is inserted inside the Singlish input
+Rationale: Input includes words such as 'app'
+Rationale: Input includes 'am'</t>
         </is>
       </c>
     </row>
@@ -2565,12 +2726,20 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats, English digital terms in Singlish</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, English Digital Terms in Singlish, Platform/App Names in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing, Extended messages with multiple sentences</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., ?; Rationale: Single words such as Postman, proper inserted; Rationale: Consecutive English words such as "oya dannawada API"; Rationale: Includes slang such as machan, thiyanawa; Rationale: Contains time format; Rationale: Includes words such as api</t>
+          <t>Evidence: "machan, oya dannawada API eka test karanna best tool ekak?"
+Rationale: It uses punctuation such as ,, ., ?
+Rationale: Single words such as 'machan, oya, dannawada, API' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "oya dannawada API" is inserted inside the Singlish input
+Rationale: Input includes words such as 'api'
+Rationale: Input includes words such as 'postman'
+Rationale: Input includes 'am'
+Rationale: Input includes 'machan, thiyanawa'
+Rationale: Long input with multiple sentences</t>
         </is>
       </c>
     </row>
@@ -2607,12 +2776,18 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Question forms, Inputs with punctuation marks, Isolated English word insertions, Multi-word English phrases in Singlish, Inputs with slang and casual phrasing, Inputs with time formats</t>
+          <t>Question forms, Inputs with punctuation marks, Isolated English Word Insertions in Singlish, Multi-Word English Phrases in Singlish, Inputs with Time Formats, Inputs with Slang and Casual Phrasing, Extended messages with multiple sentences</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>Evidence: Input contains question mark; Rationale: Uses punctuation such as ,, ., :, ?; Rationale: Single words such as Mama, dapu inserted; Rationale: Consecutive English words such as "ta office giya"; Rationale: Includes slang such as ado, puluwanda; Rationale: Contains time format</t>
+          <t>Evidence: "Ado nang, mama ada 9:00AM ta office giya. HR kiwwa IT team ekata new laptop 2 dapu kiyala. Budget eka LKR 150,000 kiyala kiwwa. Mama heta baladaganna one kochcharata order karanna one kiyala. Oya help karanda puluwanda?"
+Rationale: It uses punctuation such as ,, ., :, ?
+Rationale: Single words such as 'Ado, nang, mama, ada' are inserted in between Singlish text
+Rationale: Two or more consecutive English words such as "ta office giya" is inserted inside the Singlish input
+Rationale: Input includes 'am'
+Rationale: Input includes 'ado, puluwanda'
+Rationale: Long input with multiple sentences</t>
         </is>
       </c>
     </row>

</xml_diff>